<commit_message>
feat: semana de prueba antes del Bloque 1
Del 19 al 25 de octubre se entrena sin apuntar: Hoy muestra el día que toca
según el día de la semana, cómo buscar el peso (2 series de 12-15, RIR 3) y la
ficha de cada ejercicio, sin botón de empezar. Desde el 26 empieza la semana 1.
Plan y calendario marcan la semana de prueba. El móvil que ya tenga el perfil
creado recibe el plan nuevo (rev 2) mientras no haya entrenos apuntados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/tests/fixtures/madre-bloque1.xlsx
+++ b/web/tests/fixtures/madre-bloque1.xlsx
@@ -26,7 +26,7 @@
     <t xml:space="preserve">TU GUÍA DE GIMNASIO - BLOQUE 1 (semanas 1-4)</t>
   </si>
   <si>
-    <t xml:space="preserve">Empiezas el lunes 19 de octubre. Lunes y jueves torso, martes y viernes pierna y glúteo, con 20-30 minutos de cinta al terminar. Miércoles, sábado y domingo, descanso (caminar sí cuenta). Objetivo: más energía, menos grasa y un cuerpo más firme y fuerte.</t>
+    <t xml:space="preserve">Del 19 al 25 de octubre, semana de prueba: entrenas sin apuntar nada. Desde el lunes 26, semanas 1-4, apuntando cada entreno. Lunes y jueves torso, martes y viernes pierna y glúteo, con 20-30 minutos de cinta al terminar. Miércoles, sábado y domingo, descanso (caminar sí cuenta). Objetivo: más energía, menos grasa y un cuerpo más firme y fuerte.</t>
   </si>
   <si>
     <t xml:space="preserve">CÓMO FUNCIONA ESTE PLAN</t>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">  Semanas 1-2: aprender. Semanas 3-4: apretar un poco más</t>
   </si>
   <si>
-    <t xml:space="preserve">  Semanas 1 y 2: 2 series de 12-15 repeticiones, dejando unas 3 en reserva (RIR 3). Semanas 3 y 4: 3 series; en los ejercicios principales de 10-12 repeticiones, dejando unas 2 en reserva (RIR 2). RIR significa "repeticiones en reserva": las que podrías haber hecho de más con buena técnica. Se empieza suave porque los tendones y las articulaciones se adaptan más despacio que el músculo, y al empezar se progresa muy bien con poco volumen. Así evitas agujetas fuertes y lesiones, y llegas con ganas a la semana siguiente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cómo elegir el peso el primer día</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Haz una serie de calentamiento muy ligera. Después elige un peso con el que puedas hacer las repeticiones que tocan notando que las últimas cuestan, pero con la técnica intacta. Si te sobran más de 4 repeticiones, sube una placa. Si no llegas al mínimo, baja una. Apunta ese peso en la columna gris "Peso de partida": será tu referencia para ver cuánto has avanzado al final del bloque.</t>
+    <t xml:space="preserve">  Después de la semana de prueba: semanas 1 y 2, 2 series de 12-15 repeticiones, dejando unas 3 en reserva (RIR 3). Semanas 3 y 4: 3 series; en los ejercicios principales de 10-12 repeticiones, dejando unas 2 en reserva (RIR 2). RIR significa "repeticiones en reserva": las que podrías haber hecho de más con buena técnica. Se empieza suave porque los tendones y las articulaciones se adaptan más despacio que el músculo, y al empezar se progresa muy bien con poco volumen. Así evitas agujetas fuertes y lesiones, y llegas con ganas a la semana siguiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Semana de prueba: del 19 al 25 de octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  La primera semana haces los 4 días completos, pero sin apuntar nada: sirve para aprender las máquinas, encontrar tu peso y ver si algún ejercicio molesta el brazo. En cada ejercicio haz una serie de calentamiento muy ligera y luego 2 series de 12-15 repeticiones. Busca un peso con el que las últimas repeticiones cuesten, pero con la técnica perfecta y dejando unas 3 en reserva. Si te sobran más, sube una placa en la siguiente serie; si no llegas a 12, baja una. Si un ejercicio molesta más de 3 sobre 10, déjalo y coméntalo. El lunes 26 empiezas la semana 1 con el peso que hayas encontrado, y desde ahí ya apuntas todo.</t>
   </si>
   <si>
     <t xml:space="preserve">  Cuándo subir de peso</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Agarre / nota</t>
   </si>
   <si>
-    <t xml:space="preserve">PESO DE PARTIDA (1er día)</t>
+    <t xml:space="preserve">PRUEBA (19-25 oct) · no se apunta</t>
   </si>
   <si>
     <t xml:space="preserve">SEMANA 1</t>
@@ -191,7 +191,7 @@
     <t xml:space="preserve">Enrolla el tronco acercando las costillas a la cadera. No tires con los brazos.</t>
   </si>
   <si>
-    <t xml:space="preserve">La columna gris 'Peso de partida' es tu referencia: apunta ahí el peso que elijas el primer día que hagas cada ejercicio, y al final del bloque verás cuánto has subido. Rellena Peso, Reps y RIR de cada semana. Si en todas las series llegas al máximo de repeticiones con buena técnica -&gt; sube el peso la semana siguiente (torso: +1-2,5 kg / pierna: +2,5-5 kg). Si no, repite el mismo peso e intenta hacer 1 repetición más. Semanas 1-2: 2 series dejando 3 repeticiones en reserva (RIR 3). Semanas 3-4: 3 series (el remo, 3-4) dejando 2 (RIR 2). Si el brazo molesta más de 3 sobre 10, para ese ejercicio.</t>
+    <t xml:space="preserve">La columna gris es la semana de prueba (19-25 de octubre): esa semana no se apunta nada, solo pruebas pesos y ves si algún ejercicio molesta. Desde el lunes 26 rellena Peso, Reps y RIR de cada semana. Si en todas las series llegas al máximo de repeticiones con buena técnica -&gt; sube el peso la semana siguiente (torso: +1-2,5 kg / pierna: +2,5-5 kg). Si no, repite el mismo peso e intenta hacer 1 repetición más. Semanas 1-2: 2 series dejando 3 repeticiones en reserva (RIR 3). Semanas 3-4: 3 series (el remo, 3-4) dejando 2 (RIR 2). Si el brazo molesta más de 3 sobre 10, para ese ejercicio.</t>
   </si>
   <si>
     <t xml:space="preserve">DIA 2 - MARTES</t>
@@ -1014,7 +1014,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" ht="88" customHeight="1">
+    <row r="18" ht="101" customHeight="1">
       <c r="B18" s="16" t="s">
         <v>10</v>
       </c>
@@ -1027,7 +1027,7 @@
       <c r="D20" s="14"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" ht="75" customHeight="1">
+    <row r="21" ht="114" customHeight="1">
       <c r="B21" s="16" t="s">
         <v>12</v>
       </c>
@@ -1483,7 +1483,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="66" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -1856,7 +1856,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="66" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -2229,7 +2229,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="66" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -2602,7 +2602,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="66" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
feat: el Bloque 1 de la madre empieza una semana más tarde
Semana de prueba del 26 de octubre al 1 de noviembre y semana 1 desde el
2 de noviembre. Excel regenerado con las fechas nuevas (y su generador al
repo). rev 3 para actualizar el móvil si aún no ha apuntado nada. App 1.7.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/tests/fixtures/madre-bloque1.xlsx
+++ b/web/tests/fixtures/madre-bloque1.xlsx
@@ -26,7 +26,7 @@
     <t xml:space="preserve">TU GUÍA DE GIMNASIO - BLOQUE 1 (semanas 1-4)</t>
   </si>
   <si>
-    <t xml:space="preserve">Del 19 al 25 de octubre, semana de prueba: entrenas sin apuntar nada. Desde el lunes 26, semanas 1-4, apuntando cada entreno. Lunes y jueves torso, martes y viernes pierna y glúteo, con 20-30 minutos de cinta al terminar. Miércoles, sábado y domingo, descanso (caminar sí cuenta). Objetivo: más energía, menos grasa y un cuerpo más firme y fuerte.</t>
+    <t xml:space="preserve">Del 26 de octubre al 1 de noviembre, semana de prueba: entrenas sin apuntar nada. Desde el lunes 2 de noviembre, semanas 1-4, apuntando cada entreno. Lunes y jueves torso, martes y viernes pierna y glúteo, con 20-30 minutos de cinta al terminar. Miércoles, sábado y domingo, descanso (caminar sí cuenta). Objetivo: más energía, menos grasa y un cuerpo más firme y fuerte.</t>
   </si>
   <si>
     <t xml:space="preserve">CÓMO FUNCIONA ESTE PLAN</t>
@@ -56,10 +56,10 @@
     <t xml:space="preserve">  Después de la semana de prueba: semanas 1 y 2, 2 series de 12-15 repeticiones, dejando unas 3 en reserva (RIR 3). Semanas 3 y 4: 3 series; en los ejercicios principales de 10-12 repeticiones, dejando unas 2 en reserva (RIR 2). RIR significa "repeticiones en reserva": las que podrías haber hecho de más con buena técnica. Se empieza suave porque los tendones y las articulaciones se adaptan más despacio que el músculo, y al empezar se progresa muy bien con poco volumen. Así evitas agujetas fuertes y lesiones, y llegas con ganas a la semana siguiente.</t>
   </si>
   <si>
-    <t xml:space="preserve">  Semana de prueba: del 19 al 25 de octubre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  La primera semana haces los 4 días completos, pero sin apuntar nada: sirve para aprender las máquinas, encontrar tu peso y ver si algún ejercicio molesta el brazo. En cada ejercicio haz una serie de calentamiento muy ligera y luego 2 series de 12-15 repeticiones. Busca un peso con el que las últimas repeticiones cuesten, pero con la técnica perfecta y dejando unas 3 en reserva. Si te sobran más, sube una placa en la siguiente serie; si no llegas a 12, baja una. Si un ejercicio molesta más de 3 sobre 10, déjalo y coméntalo. El lunes 26 empiezas la semana 1 con el peso que hayas encontrado, y desde ahí ya apuntas todo.</t>
+    <t xml:space="preserve">  Semana de prueba: del 26 de octubre al 1 de noviembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  La primera semana haces los 4 días completos, pero sin apuntar nada: sirve para aprender las máquinas, encontrar tu peso y ver si algún ejercicio molesta el brazo. En cada ejercicio haz una serie de calentamiento muy ligera y luego 2 series de 12-15 repeticiones. Busca un peso con el que las últimas repeticiones cuesten, pero con la técnica perfecta y dejando unas 3 en reserva. Si te sobran más, sube una placa en la siguiente serie; si no llegas a 12, baja una. Si un ejercicio molesta más de 3 sobre 10, déjalo y coméntalo. El lunes 2 de noviembre empiezas la semana 1 con el peso que hayas encontrado, y desde ahí ya apuntas todo.</t>
   </si>
   <si>
     <t xml:space="preserve">  Cuándo subir de peso</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Agarre / nota</t>
   </si>
   <si>
-    <t xml:space="preserve">PRUEBA (19-25 oct) · no se apunta</t>
+    <t xml:space="preserve">PRUEBA (26 oct-1 nov)</t>
   </si>
   <si>
     <t xml:space="preserve">SEMANA 1</t>
@@ -191,7 +191,7 @@
     <t xml:space="preserve">Enrolla el tronco acercando las costillas a la cadera. No tires con los brazos.</t>
   </si>
   <si>
-    <t xml:space="preserve">La columna gris es la semana de prueba (19-25 de octubre): esa semana no se apunta nada, solo pruebas pesos y ves si algún ejercicio molesta. Desde el lunes 26 rellena Peso, Reps y RIR de cada semana. Si en todas las series llegas al máximo de repeticiones con buena técnica -&gt; sube el peso la semana siguiente (torso: +1-2,5 kg / pierna: +2,5-5 kg). Si no, repite el mismo peso e intenta hacer 1 repetición más. Semanas 1-2: 2 series dejando 3 repeticiones en reserva (RIR 3). Semanas 3-4: 3 series (el remo, 3-4) dejando 2 (RIR 2). Si el brazo molesta más de 3 sobre 10, para ese ejercicio.</t>
+    <t xml:space="preserve">La columna gris es la semana de prueba (del 26 de octubre al 1 de noviembre): esa semana no se apunta nada, solo pruebas pesos y ves si algún ejercicio molesta. Desde el lunes 2 de noviembre rellena Peso, Reps y RIR de cada semana. Si en todas las series llegas al máximo de repeticiones con buena técnica -&gt; sube el peso la semana siguiente (torso: +1-2,5 kg / pierna: +2,5-5 kg). Si no, repite el mismo peso e intenta hacer 1 repetición más. Semanas 1-2: 2 series dejando 3 repeticiones en reserva (RIR 3). Semanas 3-4: 3 series (el remo, 3-4) dejando 2 (RIR 2). Si el brazo molesta más de 3 sobre 10, para ese ejercicio.</t>
   </si>
   <si>
     <t xml:space="preserve">DIA 2 - MARTES</t>
@@ -952,7 +952,7 @@
       <c r="F3" s="7"/>
       <c r="G3" s="8"/>
     </row>
-    <row r="4" ht="33.0" customHeight="1">
+    <row r="4" ht="48.0" customHeight="1">
       <c r="B4" s="9" t="s">
         <v>1</v>
       </c>
@@ -1483,7 +1483,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -1856,7 +1856,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -2229,7 +2229,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>
@@ -2602,7 +2602,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="34"/>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="36" t="s">
         <v>56</v>
       </c>

</xml_diff>